<commit_message>
Seperated out line rendering functions into line_renderer.cpp, and cleaned up physics functions with AABB class
</commit_message>
<xml_diff>
--- a/UCSG - Planner.xlsx
+++ b/UCSG - Planner.xlsx
@@ -1,11 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30224"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A45372E9-A033-41BF-995E-092809A3D052}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\conno\Desktop\UCSG\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58350D39-D141-4EAD-9513-593640BEB6F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2685" yWindow="2685" windowWidth="28800" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -109,7 +114,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -353,114 +358,114 @@
   </cellStyleXfs>
   <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1">
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
           <xfpb:xfComplement i="0"/>
         </ext>
       </extLst>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1">
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
           <xfpb:xfComplement i="0"/>
         </ext>
       </extLst>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1">
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
           <xfpb:xfComplement i="0"/>
         </ext>
       </extLst>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -497,9 +502,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -537,7 +542,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -643,7 +648,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -785,7 +790,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -794,530 +799,547 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:R16"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="16.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18">
-      <c r="A1" s="18" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="19"/>
-      <c r="C1" s="19"/>
-      <c r="D1" s="19"/>
-      <c r="E1" s="19"/>
-      <c r="F1" s="19"/>
-      <c r="G1" s="19"/>
-      <c r="H1" s="19"/>
-      <c r="I1" s="19"/>
-      <c r="J1" s="19"/>
-      <c r="K1" s="19"/>
-      <c r="L1" s="19"/>
-      <c r="M1" s="19"/>
-      <c r="N1" s="19"/>
-      <c r="O1" s="19"/>
-      <c r="P1" s="19"/>
-      <c r="Q1" s="19"/>
-      <c r="R1" s="20"/>
-    </row>
-    <row r="2" spans="1:18">
-      <c r="A2" s="21"/>
-      <c r="B2" s="17"/>
-      <c r="C2" s="17"/>
-      <c r="D2" s="17"/>
-      <c r="E2" s="17"/>
-      <c r="F2" s="17"/>
-      <c r="G2" s="17"/>
-      <c r="H2" s="17"/>
-      <c r="I2" s="17"/>
-      <c r="J2" s="17"/>
-      <c r="K2" s="17"/>
-      <c r="L2" s="17"/>
-      <c r="M2" s="17"/>
-      <c r="N2" s="17"/>
-      <c r="O2" s="17"/>
-      <c r="P2" s="17"/>
-      <c r="Q2" s="17"/>
-      <c r="R2" s="22"/>
-    </row>
-    <row r="3" spans="1:18">
-      <c r="A3" s="23" t="s">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A1" s="26" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="27"/>
+      <c r="C1" s="27"/>
+      <c r="D1" s="27"/>
+      <c r="E1" s="27"/>
+      <c r="F1" s="27"/>
+      <c r="G1" s="27"/>
+      <c r="H1" s="27"/>
+      <c r="I1" s="27"/>
+      <c r="J1" s="27"/>
+      <c r="K1" s="27"/>
+      <c r="L1" s="27"/>
+      <c r="M1" s="27"/>
+      <c r="N1" s="27"/>
+      <c r="O1" s="27"/>
+      <c r="P1" s="27"/>
+      <c r="Q1" s="27"/>
+      <c r="R1" s="28"/>
+    </row>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A2" s="29"/>
+      <c r="B2" s="30"/>
+      <c r="C2" s="30"/>
+      <c r="D2" s="30"/>
+      <c r="E2" s="30"/>
+      <c r="F2" s="30"/>
+      <c r="G2" s="30"/>
+      <c r="H2" s="30"/>
+      <c r="I2" s="30"/>
+      <c r="J2" s="30"/>
+      <c r="K2" s="30"/>
+      <c r="L2" s="30"/>
+      <c r="M2" s="30"/>
+      <c r="N2" s="30"/>
+      <c r="O2" s="30"/>
+      <c r="P2" s="30"/>
+      <c r="Q2" s="30"/>
+      <c r="R2" s="31"/>
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A3" s="35" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="24"/>
-      <c r="C3" s="24"/>
-      <c r="D3" s="24"/>
-      <c r="E3" s="24"/>
-      <c r="F3" s="24"/>
-      <c r="G3" s="25" t="s">
+      <c r="B3" s="36"/>
+      <c r="C3" s="36"/>
+      <c r="D3" s="36"/>
+      <c r="E3" s="36"/>
+      <c r="F3" s="36"/>
+      <c r="G3" s="37" t="s">
         <v>2</v>
       </c>
-      <c r="H3" s="26"/>
-      <c r="I3" s="26"/>
-      <c r="J3" s="26"/>
-      <c r="K3" s="26"/>
-      <c r="L3" s="27"/>
-      <c r="M3" s="28" t="s">
+      <c r="H3" s="38"/>
+      <c r="I3" s="38"/>
+      <c r="J3" s="38"/>
+      <c r="K3" s="38"/>
+      <c r="L3" s="39"/>
+      <c r="M3" s="40" t="s">
         <v>3</v>
       </c>
-      <c r="N3" s="28"/>
-      <c r="O3" s="28"/>
-      <c r="P3" s="28"/>
-      <c r="Q3" s="28"/>
-      <c r="R3" s="29"/>
-    </row>
-    <row r="4" spans="1:18">
-      <c r="A4" s="1" t="s">
+      <c r="N3" s="40"/>
+      <c r="O3" s="40"/>
+      <c r="P3" s="40"/>
+      <c r="Q3" s="40"/>
+      <c r="R3" s="41"/>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A4" s="23" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="2"/>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
-      <c r="F4" s="3"/>
-      <c r="G4" s="4" t="s">
+      <c r="B4" s="24"/>
+      <c r="C4" s="24"/>
+      <c r="D4" s="24"/>
+      <c r="E4" s="24"/>
+      <c r="F4" s="25"/>
+      <c r="G4" s="32" t="s">
         <v>4</v>
       </c>
-      <c r="H4" s="5"/>
-      <c r="I4" s="5"/>
-      <c r="J4" s="5"/>
-      <c r="K4" s="5"/>
-      <c r="L4" s="6"/>
-      <c r="M4" s="4" t="s">
+      <c r="H4" s="33"/>
+      <c r="I4" s="33"/>
+      <c r="J4" s="33"/>
+      <c r="K4" s="33"/>
+      <c r="L4" s="34"/>
+      <c r="M4" s="32" t="s">
         <v>4</v>
       </c>
-      <c r="N4" s="5"/>
-      <c r="O4" s="5"/>
-      <c r="P4" s="5"/>
-      <c r="Q4" s="5"/>
-      <c r="R4" s="6"/>
-    </row>
-    <row r="5" spans="1:18">
-      <c r="A5" s="32" t="s">
+      <c r="N4" s="33"/>
+      <c r="O4" s="33"/>
+      <c r="P4" s="33"/>
+      <c r="Q4" s="33"/>
+      <c r="R4" s="34"/>
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A5" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="34" t="s">
+      <c r="B5" s="17" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="33"/>
-      <c r="D5" s="33"/>
-      <c r="E5" s="33"/>
-      <c r="F5" s="35"/>
-      <c r="G5" s="32" t="s">
+      <c r="C5" s="18"/>
+      <c r="D5" s="18"/>
+      <c r="E5" s="18"/>
+      <c r="F5" s="19"/>
+      <c r="G5" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="H5" s="36" t="s">
+      <c r="H5" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="I5" s="37"/>
-      <c r="J5" s="37"/>
-      <c r="K5" s="37"/>
-      <c r="L5" s="38"/>
-      <c r="M5" s="32" t="s">
+      <c r="I5" s="21"/>
+      <c r="J5" s="21"/>
+      <c r="K5" s="21"/>
+      <c r="L5" s="22"/>
+      <c r="M5" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="N5" s="34" t="s">
+      <c r="N5" s="17" t="s">
         <v>6</v>
       </c>
-      <c r="O5" s="33"/>
-      <c r="P5" s="33"/>
-      <c r="Q5" s="33"/>
-      <c r="R5" s="35"/>
-    </row>
-    <row r="6" spans="1:18">
-      <c r="A6" s="30">
+      <c r="O5" s="18"/>
+      <c r="P5" s="18"/>
+      <c r="Q5" s="18"/>
+      <c r="R5" s="19"/>
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A6" s="5">
         <v>1</v>
       </c>
-      <c r="B6" s="16" t="s">
+      <c r="B6" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="15"/>
-      <c r="D6" s="15"/>
-      <c r="E6" s="15"/>
-      <c r="F6" s="39" t="b">
-        <v>0</v>
-      </c>
-      <c r="G6" s="11">
+      <c r="C6" s="16"/>
+      <c r="D6" s="16"/>
+      <c r="E6" s="16"/>
+      <c r="F6" s="8" t="b">
+        <v>0</v>
+      </c>
+      <c r="G6" s="1">
         <v>1</v>
       </c>
-      <c r="H6" s="36" t="s">
+      <c r="H6" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="I6" s="37"/>
-      <c r="J6" s="37"/>
-      <c r="K6" s="37"/>
-      <c r="L6" s="39" t="b">
-        <v>0</v>
-      </c>
-      <c r="M6" s="12">
+      <c r="I6" s="21"/>
+      <c r="J6" s="21"/>
+      <c r="K6" s="21"/>
+      <c r="L6" s="8" t="b">
+        <v>0</v>
+      </c>
+      <c r="M6" s="3">
         <v>1</v>
       </c>
-      <c r="N6" s="16" t="s">
+      <c r="N6" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="O6" s="15"/>
-      <c r="P6" s="15"/>
-      <c r="Q6" s="15"/>
-      <c r="R6" s="39" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:18">
-      <c r="A7" s="30">
+      <c r="O6" s="16"/>
+      <c r="P6" s="16"/>
+      <c r="Q6" s="16"/>
+      <c r="R6" s="8" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A7" s="5">
         <v>2</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="B7" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="C7" s="8"/>
-      <c r="D7" s="8"/>
-      <c r="E7" s="8"/>
-      <c r="F7" s="40" t="b">
-        <v>0</v>
-      </c>
-      <c r="G7" s="11">
+      <c r="C7" s="12"/>
+      <c r="D7" s="12"/>
+      <c r="E7" s="12"/>
+      <c r="F7" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="G7" s="1">
         <v>2</v>
       </c>
-      <c r="H7" s="7" t="s">
+      <c r="H7" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="I7" s="8"/>
-      <c r="J7" s="8"/>
-      <c r="K7" s="8"/>
-      <c r="L7" s="40" t="b">
-        <v>0</v>
-      </c>
-      <c r="M7" s="12">
+      <c r="I7" s="12"/>
+      <c r="J7" s="12"/>
+      <c r="K7" s="12"/>
+      <c r="L7" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="M7" s="3">
         <v>2</v>
       </c>
-      <c r="N7" s="7" t="s">
+      <c r="N7" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="O7" s="8"/>
-      <c r="P7" s="8"/>
-      <c r="Q7" s="8"/>
-      <c r="R7" s="40" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:18">
-      <c r="A8" s="30">
+      <c r="O7" s="12"/>
+      <c r="P7" s="12"/>
+      <c r="Q7" s="12"/>
+      <c r="R7" s="9" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A8" s="5">
         <v>3</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="B8" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="C8" s="8"/>
-      <c r="D8" s="8"/>
-      <c r="E8" s="8"/>
-      <c r="F8" s="40" t="b">
-        <v>0</v>
-      </c>
-      <c r="G8" s="11">
+      <c r="C8" s="12"/>
+      <c r="D8" s="12"/>
+      <c r="E8" s="12"/>
+      <c r="F8" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="G8" s="1">
         <v>3</v>
       </c>
-      <c r="H8" s="7" t="s">
+      <c r="H8" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="I8" s="8"/>
-      <c r="J8" s="8"/>
-      <c r="K8" s="8"/>
-      <c r="L8" s="40" t="b">
-        <v>0</v>
-      </c>
-      <c r="M8" s="12">
+      <c r="I8" s="12"/>
+      <c r="J8" s="12"/>
+      <c r="K8" s="12"/>
+      <c r="L8" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="M8" s="3">
         <v>3</v>
       </c>
-      <c r="N8" s="7" t="s">
+      <c r="N8" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="O8" s="8"/>
-      <c r="P8" s="8"/>
-      <c r="Q8" s="8"/>
-      <c r="R8" s="40" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:18">
-      <c r="A9" s="30">
+      <c r="O8" s="12"/>
+      <c r="P8" s="12"/>
+      <c r="Q8" s="12"/>
+      <c r="R8" s="9" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A9" s="5">
         <v>4</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="B9" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="C9" s="8"/>
-      <c r="D9" s="8"/>
-      <c r="E9" s="8"/>
-      <c r="F9" s="40" t="b">
-        <v>0</v>
-      </c>
-      <c r="G9" s="11">
+      <c r="C9" s="12"/>
+      <c r="D9" s="12"/>
+      <c r="E9" s="12"/>
+      <c r="F9" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="G9" s="1">
         <v>4</v>
       </c>
-      <c r="H9" s="7" t="s">
+      <c r="H9" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="I9" s="8"/>
-      <c r="J9" s="8"/>
-      <c r="K9" s="8"/>
-      <c r="L9" s="40" t="b">
-        <v>0</v>
-      </c>
-      <c r="M9" s="12">
+      <c r="I9" s="12"/>
+      <c r="J9" s="12"/>
+      <c r="K9" s="12"/>
+      <c r="L9" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="M9" s="3">
         <v>4</v>
       </c>
-      <c r="N9" s="7" t="s">
+      <c r="N9" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="O9" s="8"/>
-      <c r="P9" s="8"/>
-      <c r="Q9" s="8"/>
-      <c r="R9" s="40" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:18">
-      <c r="A10" s="30">
+      <c r="O9" s="12"/>
+      <c r="P9" s="12"/>
+      <c r="Q9" s="12"/>
+      <c r="R9" s="9" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A10" s="5">
         <v>5</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="B10" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="C10" s="8"/>
-      <c r="D10" s="8"/>
-      <c r="E10" s="8"/>
-      <c r="F10" s="40" t="b">
-        <v>0</v>
-      </c>
-      <c r="G10" s="11">
+      <c r="C10" s="12"/>
+      <c r="D10" s="12"/>
+      <c r="E10" s="12"/>
+      <c r="F10" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="G10" s="1">
         <v>5</v>
       </c>
-      <c r="H10" s="7" t="s">
+      <c r="H10" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="I10" s="8"/>
-      <c r="J10" s="8"/>
-      <c r="K10" s="8"/>
-      <c r="L10" s="40" t="b">
-        <v>0</v>
-      </c>
-      <c r="M10" s="12">
+      <c r="I10" s="12"/>
+      <c r="J10" s="12"/>
+      <c r="K10" s="12"/>
+      <c r="L10" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="M10" s="3">
         <v>5</v>
       </c>
-      <c r="N10" s="7" t="s">
+      <c r="N10" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="O10" s="8"/>
-      <c r="P10" s="8"/>
-      <c r="Q10" s="8"/>
-      <c r="R10" s="40" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:18">
-      <c r="A11" s="30">
+      <c r="O10" s="12"/>
+      <c r="P10" s="12"/>
+      <c r="Q10" s="12"/>
+      <c r="R10" s="9" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A11" s="5">
         <v>6</v>
       </c>
-      <c r="B11" s="7" t="s">
+      <c r="B11" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="C11" s="8"/>
-      <c r="D11" s="8"/>
-      <c r="E11" s="8"/>
-      <c r="F11" s="40" t="b">
-        <v>0</v>
-      </c>
-      <c r="G11" s="11">
+      <c r="C11" s="12"/>
+      <c r="D11" s="12"/>
+      <c r="E11" s="12"/>
+      <c r="F11" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="G11" s="1">
         <v>6</v>
       </c>
-      <c r="H11" s="7"/>
-      <c r="I11" s="8"/>
-      <c r="J11" s="8"/>
-      <c r="K11" s="8"/>
-      <c r="L11" s="40" t="b">
-        <v>0</v>
-      </c>
-      <c r="M11" s="12">
+      <c r="H11" s="11"/>
+      <c r="I11" s="12"/>
+      <c r="J11" s="12"/>
+      <c r="K11" s="12"/>
+      <c r="L11" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="M11" s="3">
         <v>6</v>
       </c>
-      <c r="N11" s="7"/>
-      <c r="O11" s="8"/>
-      <c r="P11" s="8"/>
-      <c r="Q11" s="8"/>
-      <c r="R11" s="40" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:18">
-      <c r="A12" s="30">
+      <c r="N11" s="11"/>
+      <c r="O11" s="12"/>
+      <c r="P11" s="12"/>
+      <c r="Q11" s="12"/>
+      <c r="R11" s="9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A12" s="5">
         <v>7</v>
       </c>
-      <c r="B12" s="7" t="s">
+      <c r="B12" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="C12" s="8"/>
-      <c r="D12" s="8"/>
-      <c r="E12" s="8"/>
-      <c r="F12" s="40" t="b">
-        <v>0</v>
-      </c>
-      <c r="G12" s="11">
+      <c r="C12" s="12"/>
+      <c r="D12" s="12"/>
+      <c r="E12" s="12"/>
+      <c r="F12" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="G12" s="1">
         <v>7</v>
       </c>
-      <c r="H12" s="7"/>
-      <c r="I12" s="8"/>
-      <c r="J12" s="8"/>
-      <c r="K12" s="8"/>
-      <c r="L12" s="40" t="b">
-        <v>0</v>
-      </c>
-      <c r="M12" s="12">
+      <c r="H12" s="11"/>
+      <c r="I12" s="12"/>
+      <c r="J12" s="12"/>
+      <c r="K12" s="12"/>
+      <c r="L12" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="M12" s="3">
         <v>7</v>
       </c>
-      <c r="N12" s="7"/>
-      <c r="O12" s="8"/>
-      <c r="P12" s="8"/>
-      <c r="Q12" s="8"/>
-      <c r="R12" s="40" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:18">
-      <c r="A13" s="30">
+      <c r="N12" s="11"/>
+      <c r="O12" s="12"/>
+      <c r="P12" s="12"/>
+      <c r="Q12" s="12"/>
+      <c r="R12" s="9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A13" s="5">
         <v>8</v>
       </c>
-      <c r="B13" s="7"/>
-      <c r="C13" s="8"/>
-      <c r="D13" s="8"/>
-      <c r="E13" s="8"/>
-      <c r="F13" s="40" t="b">
-        <v>0</v>
-      </c>
-      <c r="G13" s="11">
+      <c r="B13" s="11"/>
+      <c r="C13" s="12"/>
+      <c r="D13" s="12"/>
+      <c r="E13" s="12"/>
+      <c r="F13" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="G13" s="1">
         <v>8</v>
       </c>
-      <c r="H13" s="7"/>
-      <c r="I13" s="8"/>
-      <c r="J13" s="8"/>
-      <c r="K13" s="8"/>
-      <c r="L13" s="40" t="b">
-        <v>0</v>
-      </c>
-      <c r="M13" s="12">
+      <c r="H13" s="11"/>
+      <c r="I13" s="12"/>
+      <c r="J13" s="12"/>
+      <c r="K13" s="12"/>
+      <c r="L13" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="M13" s="3">
         <v>8</v>
       </c>
-      <c r="N13" s="7"/>
-      <c r="O13" s="8"/>
-      <c r="P13" s="8"/>
-      <c r="Q13" s="8"/>
-      <c r="R13" s="40" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:18">
-      <c r="A14" s="30">
+      <c r="N13" s="11"/>
+      <c r="O13" s="12"/>
+      <c r="P13" s="12"/>
+      <c r="Q13" s="12"/>
+      <c r="R13" s="9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A14" s="5">
         <v>9</v>
       </c>
-      <c r="B14" s="7"/>
-      <c r="C14" s="8"/>
-      <c r="D14" s="8"/>
-      <c r="E14" s="8"/>
-      <c r="F14" s="40" t="b">
-        <v>0</v>
-      </c>
-      <c r="G14" s="11">
+      <c r="B14" s="11"/>
+      <c r="C14" s="12"/>
+      <c r="D14" s="12"/>
+      <c r="E14" s="12"/>
+      <c r="F14" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="G14" s="1">
         <v>9</v>
       </c>
-      <c r="H14" s="7"/>
-      <c r="I14" s="8"/>
-      <c r="J14" s="8"/>
-      <c r="K14" s="8"/>
-      <c r="L14" s="40" t="b">
-        <v>0</v>
-      </c>
-      <c r="M14" s="12">
+      <c r="H14" s="11"/>
+      <c r="I14" s="12"/>
+      <c r="J14" s="12"/>
+      <c r="K14" s="12"/>
+      <c r="L14" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="M14" s="3">
         <v>9</v>
       </c>
-      <c r="N14" s="7"/>
-      <c r="O14" s="8"/>
-      <c r="P14" s="8"/>
-      <c r="Q14" s="8"/>
-      <c r="R14" s="40" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:18">
-      <c r="A15" s="30">
+      <c r="N14" s="11"/>
+      <c r="O14" s="12"/>
+      <c r="P14" s="12"/>
+      <c r="Q14" s="12"/>
+      <c r="R14" s="9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A15" s="5">
         <v>10</v>
       </c>
-      <c r="B15" s="7"/>
-      <c r="C15" s="8"/>
-      <c r="D15" s="8"/>
-      <c r="E15" s="8"/>
-      <c r="F15" s="40" t="b">
-        <v>0</v>
-      </c>
-      <c r="G15" s="11">
+      <c r="B15" s="11"/>
+      <c r="C15" s="12"/>
+      <c r="D15" s="12"/>
+      <c r="E15" s="12"/>
+      <c r="F15" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="G15" s="1">
         <v>10</v>
       </c>
-      <c r="H15" s="7"/>
-      <c r="I15" s="8"/>
-      <c r="J15" s="8"/>
-      <c r="K15" s="8"/>
-      <c r="L15" s="40" t="b">
-        <v>0</v>
-      </c>
-      <c r="M15" s="12">
+      <c r="H15" s="11"/>
+      <c r="I15" s="12"/>
+      <c r="J15" s="12"/>
+      <c r="K15" s="12"/>
+      <c r="L15" s="9" t="b">
+        <v>0</v>
+      </c>
+      <c r="M15" s="3">
         <v>10</v>
       </c>
-      <c r="N15" s="7"/>
-      <c r="O15" s="8"/>
-      <c r="P15" s="8"/>
-      <c r="Q15" s="8"/>
-      <c r="R15" s="40" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="1:18">
-      <c r="A16" s="31">
+      <c r="N15" s="11"/>
+      <c r="O15" s="12"/>
+      <c r="P15" s="12"/>
+      <c r="Q15" s="12"/>
+      <c r="R15" s="9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A16" s="6">
         <v>11</v>
       </c>
-      <c r="B16" s="9"/>
-      <c r="C16" s="10"/>
-      <c r="D16" s="10"/>
-      <c r="E16" s="10"/>
-      <c r="F16" s="41" t="b">
-        <v>0</v>
-      </c>
-      <c r="G16" s="13">
+      <c r="B16" s="13"/>
+      <c r="C16" s="14"/>
+      <c r="D16" s="14"/>
+      <c r="E16" s="14"/>
+      <c r="F16" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="G16" s="2">
         <v>11</v>
       </c>
-      <c r="H16" s="9"/>
-      <c r="I16" s="10"/>
-      <c r="J16" s="10"/>
-      <c r="K16" s="10"/>
-      <c r="L16" s="41" t="b">
-        <v>0</v>
-      </c>
-      <c r="M16" s="14">
+      <c r="H16" s="13"/>
+      <c r="I16" s="14"/>
+      <c r="J16" s="14"/>
+      <c r="K16" s="14"/>
+      <c r="L16" s="10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M16" s="4">
         <v>11</v>
       </c>
-      <c r="N16" s="9"/>
-      <c r="O16" s="10"/>
-      <c r="P16" s="10"/>
-      <c r="Q16" s="10"/>
-      <c r="R16" s="41" t="b">
+      <c r="N16" s="13"/>
+      <c r="O16" s="14"/>
+      <c r="P16" s="14"/>
+      <c r="Q16" s="14"/>
+      <c r="R16" s="10" t="b">
         <v>0</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="43">
-    <mergeCell ref="N12:Q12"/>
-    <mergeCell ref="N13:Q13"/>
-    <mergeCell ref="N14:Q14"/>
-    <mergeCell ref="N15:Q15"/>
-    <mergeCell ref="N16:Q16"/>
+    <mergeCell ref="B12:E12"/>
+    <mergeCell ref="A4:F4"/>
+    <mergeCell ref="A1:R2"/>
+    <mergeCell ref="G4:L4"/>
+    <mergeCell ref="M4:R4"/>
+    <mergeCell ref="B5:F5"/>
+    <mergeCell ref="A3:F3"/>
+    <mergeCell ref="G3:L3"/>
+    <mergeCell ref="M3:R3"/>
+    <mergeCell ref="H15:K15"/>
+    <mergeCell ref="H16:K16"/>
+    <mergeCell ref="N5:R5"/>
+    <mergeCell ref="H5:L5"/>
+    <mergeCell ref="H6:K6"/>
+    <mergeCell ref="H7:K7"/>
+    <mergeCell ref="H8:K8"/>
+    <mergeCell ref="H9:K9"/>
+    <mergeCell ref="H10:K10"/>
+    <mergeCell ref="H11:K11"/>
+    <mergeCell ref="H12:K12"/>
+    <mergeCell ref="H13:K13"/>
+    <mergeCell ref="H14:K14"/>
     <mergeCell ref="B13:E13"/>
     <mergeCell ref="B14:E14"/>
     <mergeCell ref="B15:E15"/>
@@ -1334,28 +1356,11 @@
     <mergeCell ref="B9:E9"/>
     <mergeCell ref="B10:E10"/>
     <mergeCell ref="B11:E11"/>
-    <mergeCell ref="H10:K10"/>
-    <mergeCell ref="H11:K11"/>
-    <mergeCell ref="H12:K12"/>
-    <mergeCell ref="H13:K13"/>
-    <mergeCell ref="H14:K14"/>
-    <mergeCell ref="H15:K15"/>
-    <mergeCell ref="H16:K16"/>
-    <mergeCell ref="N5:R5"/>
-    <mergeCell ref="H5:L5"/>
-    <mergeCell ref="H6:K6"/>
-    <mergeCell ref="H7:K7"/>
-    <mergeCell ref="H8:K8"/>
-    <mergeCell ref="H9:K9"/>
-    <mergeCell ref="B12:E12"/>
-    <mergeCell ref="A4:F4"/>
-    <mergeCell ref="A1:R2"/>
-    <mergeCell ref="G4:L4"/>
-    <mergeCell ref="M4:R4"/>
-    <mergeCell ref="B5:F5"/>
-    <mergeCell ref="A3:F3"/>
-    <mergeCell ref="G3:L3"/>
-    <mergeCell ref="M3:R3"/>
+    <mergeCell ref="N12:Q12"/>
+    <mergeCell ref="N13:Q13"/>
+    <mergeCell ref="N14:Q14"/>
+    <mergeCell ref="N15:Q15"/>
+    <mergeCell ref="N16:Q16"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>